<commit_message>
chore: add in btech,bca 62 new
</commit_message>
<xml_diff>
--- a/raw/time_tables/B.Tech 62 (btech-62)/1/1.xlsx
+++ b/raw/time_tables/B.Tech 62 (btech-62)/1/1.xlsx
@@ -1960,7 +1960,7 @@
       <c r="A19" s="11" t="n"/>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>TG2(MA111)-F10/DCS</t>
+          <t>TG2(MA111)-TS12/DCS</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
@@ -9554,7 +9554,7 @@
       </c>
       <c r="D203" s="13" t="inlineStr">
         <is>
-          <t>TA10(MA111)-F7/DGA</t>
+          <t>TA10(MA111)-F7/DCS</t>
         </is>
       </c>
       <c r="E203" s="12" t="inlineStr"/>
@@ -9862,7 +9862,7 @@
       <c r="C212" s="4" t="n"/>
       <c r="D212" s="10" t="inlineStr">
         <is>
-          <t>PA3(EC111)-BEL1/GRA,RHA</t>
+          <t>PA3(EC111)-BEL1/RDR,RHA</t>
         </is>
       </c>
       <c r="E212" s="4" t="n"/>

</xml_diff>